<commit_message>
added test case - 'Check Account Details'
</commit_message>
<xml_diff>
--- a/TestPlan.xlsx
+++ b/TestPlan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JoelJohnson(G10XIND)\Desktop\cypressFramework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCD47D5A-030F-4B07-9ED3-285EFA89108F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5C8B137-E2B6-4BEB-BE66-C56C5A9BE913}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3540" yWindow="1068" windowWidth="13008" windowHeight="9456" activeTab="1" xr2:uid="{F12E7399-85D7-4ED8-8C27-8CECEEF59108}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{F12E7399-85D7-4ED8-8C27-8CECEEF59108}"/>
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="Request Loan" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="39">
   <si>
     <t>Test Plan - Cypress Test Automation Framework on ParaBank Demo Website</t>
   </si>
@@ -274,20 +275,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -636,12 +637,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -657,10 +658,10 @@
       <c r="H2" s="2"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="9"/>
+      <c r="C3" s="12"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -789,36 +790,36 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.6640625" customWidth="1"/>
-    <col min="2" max="2" width="17.44140625" style="12" customWidth="1"/>
+    <col min="2" max="2" width="17.44140625" style="10" customWidth="1"/>
     <col min="3" max="3" width="52.88671875" customWidth="1"/>
     <col min="4" max="4" width="11.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B2" s="11"/>
+      <c r="B2" s="9"/>
       <c r="C2" s="5"/>
       <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="9"/>
+      <c r="C3" s="12"/>
       <c r="D3" s="7"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="9" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="5" t="s">
@@ -832,7 +833,7 @@
       <c r="A5">
         <v>1</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="10" t="s">
         <v>22</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -846,49 +847,55 @@
       <c r="A6">
         <v>2</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="10" t="s">
         <v>24</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="10"/>
+      <c r="D6" s="6" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="7" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>3</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="10" t="s">
         <v>26</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="10"/>
+      <c r="D7" s="6" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="8" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>4</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="10" t="s">
         <v>27</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="10"/>
+      <c r="D8" s="6" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C9" s="1"/>
-      <c r="D9" s="10"/>
+      <c r="D9" s="8"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C10" s="1"/>
-      <c r="D10" s="10"/>
+      <c r="D10" s="8"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C11" s="1"/>
-      <c r="D11" s="10"/>
+      <c r="D11" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -911,30 +918,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B2" s="11"/>
+      <c r="B2" s="9"/>
       <c r="C2" s="5"/>
       <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="9"/>
+      <c r="C3" s="12"/>
       <c r="D3" s="7"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="9" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="5" t="s">
@@ -948,49 +955,49 @@
       <c r="A5">
         <v>1</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="10" t="s">
         <v>31</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="10"/>
+      <c r="D5" s="8"/>
     </row>
     <row r="6" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="10" t="s">
         <v>33</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="10"/>
+      <c r="D6" s="8"/>
     </row>
     <row r="7" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>3</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="10" t="s">
         <v>35</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="10"/>
+      <c r="D7" s="8"/>
     </row>
     <row r="8" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>4</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="10" t="s">
         <v>37</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="10"/>
+      <c r="D8" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>